<commit_message>
Added the edit/save button in admin delete prdocut page , only can be deleted invididually and q1 to p3 can be edited"
</commit_message>
<xml_diff>
--- a/static/assets/uploads/ProductList.xlsx
+++ b/static/assets/uploads/ProductList.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ragha\Documents\NariNakhre\static\assets\uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A8D4F65-606F-4A19-BD88-EB4F7E2932A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66CE846D-AFC8-4373-BBFE-4FC12FD93591}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="29">
   <si>
     <t>sku</t>
   </si>
@@ -57,57 +57,9 @@
     <t>description</t>
   </si>
   <si>
-    <t>BNG-001</t>
-  </si>
-  <si>
-    <t>Rose Gold Bangle</t>
-  </si>
-  <si>
-    <t>Silk &amp; Metal</t>
-  </si>
-  <si>
-    <t>Rose Gold</t>
-  </si>
-  <si>
-    <t>2.4, 2.6</t>
-  </si>
-  <si>
-    <t>Jewelry</t>
-  </si>
-  <si>
     <t>Bangles</t>
   </si>
   <si>
-    <t>Hand-crafted silk bangles with premium ruby-colored stones.</t>
-  </si>
-  <si>
-    <t>BNG-002</t>
-  </si>
-  <si>
-    <t>Velvet Matte Red</t>
-  </si>
-  <si>
-    <t>Organic</t>
-  </si>
-  <si>
-    <t>Ruby Red</t>
-  </si>
-  <si>
-    <t>N/A</t>
-  </si>
-  <si>
-    <t>Beauty</t>
-  </si>
-  <si>
-    <t>Lipsticks</t>
-  </si>
-  <si>
-    <t>Long-lasting velvet finish with organic ingredients.</t>
-  </si>
-  <si>
-    <t>BNG-003</t>
-  </si>
-  <si>
     <t>quantity1</t>
   </si>
   <si>
@@ -124,16 +76,92 @@
   </si>
   <si>
     <t>price3</t>
+  </si>
+  <si>
+    <r>
+      <t>Nari Nakhre</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Vibrant Yellow Silk Thread Bangle Set with Intricate Silver Stone Studded Kada (Pack of 20)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Nari Nakhre</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Luxurious 28-Piece Bridal Chuda Set – Brass Base with Red Velvet Finish, Artificial Stones, and Pearl Embellishments</t>
+    </r>
+  </si>
+  <si>
+    <t>Elevate your bridal look with this exquisite 28-piece Chuda Set from Nari Nakhre, a brand by Mohini Cosmetics. Crafted for the modern bride who cherishes tradition, this set features a premium brass base, ensuring durability and a high-end feel. The bangles are adorned with shimmering artificial stones and delicate pearls, set against a rich red velvet-feel thread wrap. Whether it’s your wedding day, an engagement, or a grand festive celebration, this complete set for both hands adds a regal touch to your ensemble. For further details, please visit www.narinakhre.com or mail at hello@mohinicosmetics.com.</t>
+  </si>
+  <si>
+    <t>Brass</t>
+  </si>
+  <si>
+    <t>Red</t>
+  </si>
+  <si>
+    <t>2.4,2.6,2.8</t>
+  </si>
+  <si>
+    <t>Chudas</t>
+  </si>
+  <si>
+    <t>Add a splash of sunshine to your ethnic wardrobe with this stunning 20-piece bangle set by Nari Nakhre, a brand by Mohini Cosmetics. This set features a beautiful combination of bright yellow silk-thread bangles paired with high-quality silver-toned kadas heavily embellished with sparkling artificial stones. Crafted on a durable brass base, these bangles are designed for longevity and comfort. Perfect for Haldi ceremonies, festive gatherings, and weddings, this set offers a perfect blend of traditional charm and modern sparkle. For further details, please visit www.narinakhre.com or mail at hello@mohinicosmetics.com.</t>
+  </si>
+  <si>
+    <t>012025BNGMR004</t>
+  </si>
+  <si>
+    <t>012025BNGRE014</t>
+  </si>
+  <si>
+    <t>Nari Nakhre** Royal Emerald Green Silk Thread Bangle Set with Gold-Toned Stone Studded Kadas (Pack of 16)</t>
+  </si>
+  <si>
+    <t>012025BNGRE015</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -156,14 +184,24 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -477,86 +515,51 @@
         <v>9</v>
       </c>
       <c r="K1" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="L1" t="s">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="M1" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="N1" t="s">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="O1" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="P1" t="s">
-        <v>32</v>
+        <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G2" t="s">
+        <v>22</v>
+      </c>
+      <c r="H2" t="s">
         <v>10</v>
       </c>
-      <c r="B2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2">
-        <v>7117</v>
-      </c>
-      <c r="D2">
-        <v>3</v>
-      </c>
-      <c r="E2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H2" t="s">
-        <v>15</v>
-      </c>
       <c r="I2" t="s">
-        <v>16</v>
-      </c>
-      <c r="J2" t="s">
-        <v>17</v>
-      </c>
-      <c r="K2">
-        <v>100</v>
-      </c>
-      <c r="L2" s="1">
-        <v>800</v>
-      </c>
-      <c r="M2">
-        <v>45</v>
-      </c>
-      <c r="N2">
-        <v>444</v>
-      </c>
-      <c r="O2">
-        <v>54</v>
-      </c>
-      <c r="P2">
-        <v>454</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="L2" s="1"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>18</v>
-      </c>
-      <c r="B3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C3">
-        <v>7117</v>
-      </c>
-      <c r="D3">
-        <v>3</v>
       </c>
       <c r="E3" t="s">
         <v>20</v>
@@ -568,84 +571,30 @@
         <v>22</v>
       </c>
       <c r="H3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I3" t="s">
         <v>23</v>
       </c>
-      <c r="I3" t="s">
-        <v>24</v>
-      </c>
-      <c r="J3" t="s">
-        <v>25</v>
-      </c>
-      <c r="K3">
-        <v>200</v>
-      </c>
-      <c r="L3" s="1">
-        <v>4500</v>
-      </c>
-      <c r="M3">
-        <v>21</v>
-      </c>
-      <c r="N3">
-        <v>22</v>
-      </c>
-      <c r="O3">
-        <v>2121</v>
-      </c>
-      <c r="P3">
-        <v>544</v>
-      </c>
+      <c r="J3" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="L3" s="1"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C4">
-        <v>7117</v>
-      </c>
-      <c r="D4">
-        <v>3</v>
-      </c>
-      <c r="E4" t="s">
-        <v>20</v>
-      </c>
-      <c r="F4" t="s">
-        <v>21</v>
-      </c>
-      <c r="G4" t="s">
-        <v>22</v>
-      </c>
-      <c r="H4" t="s">
-        <v>23</v>
-      </c>
-      <c r="I4" t="s">
-        <v>24</v>
-      </c>
-      <c r="J4" t="s">
-        <v>25</v>
-      </c>
-      <c r="K4">
-        <v>300</v>
-      </c>
-      <c r="L4" s="1">
-        <v>4100</v>
-      </c>
-      <c r="M4">
-        <v>21</v>
-      </c>
-      <c r="N4">
-        <v>11</v>
-      </c>
-      <c r="O4">
-        <v>211</v>
-      </c>
-      <c r="P4">
-        <v>5454</v>
-      </c>
+        <v>27</v>
+      </c>
+      <c r="L4" s="1"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="J3" r:id="rId1" display="https://www.narinakhre.com/" xr:uid="{1FF903D5-2C7D-4E7E-89D2-979CAFC435E4}"/>
+    <hyperlink ref="J2" r:id="rId2" display="https://www.narinakhre.com/" xr:uid="{B84819B7-1F16-492A-9902-F6FB03EEEA8D}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>